<commit_message>
Atnaujinti AGENTO_INSTRUKCIJOS.md ir Build-ApzvalgaJson.ps1 statinei architektūrai
- SOP dabar aprašo data/problems.json kaip kanoninį šaltinį (ne Claude Artifact db)
- Build-ApzvalgaJson.ps1 skaito tiesiai iš data/problems.json
- Pašalinti pasenę tarpiniai JSON failai

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ataskaitos/VK_zin_apzvalga_2026-09-03.xlsx
+++ b/ataskaitos/VK_zin_apzvalga_2026-09-03.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="Zin. apzvalga 2026-09-03" sheetId="1" r:id="rId1"/>
+    <sheet name="Zin. apzvalga" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -118,6 +118,27 @@
     <t xml:space="preserve">Medikų trūkumas ir atlyginimų atotrūkis savivaldybių poliklinikose</t>
   </si>
   <si>
+    <t xml:space="preserve">STT nustatė korupcijos rizikas sporto infrastruktūros ir programų finansavime</t>
+  </si>
+  <si>
+    <t xml:space="preserve">„Per 2023–2025 m. iš valstybės biudžeto sporto finansavimui skirta daugiau kaip 76,6 mln. eurų.“ STT korupcijos rizikos analizė apėmė Švietimo, mokslo ir sporto ministeriją, Nacionalinę sporto agentūrą ir Vilniaus, Panevėžio, Kauno, Akmenės, Kupiškio bei Plungės savivaldybes. „Finansavimas skirtas futbolo klubui, kurio prezidentas buvo savivaldybės meras.“ Valstybės investuota baseinų infrastruktūra „naudojama ir komercinėmis SPA ar pirčių paslaugomis“ be aiškių viešojo intereso sąlygų.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jp.lt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jp.lt straipsnis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-06-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Švietimas, mokslas ir sportas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sporto finansavimo skaidrumas ir interesų konfliktai</t>
+  </si>
+  <si>
     <t xml:space="preserve">Prognozuojamas iki 6000 mokytojų trūkumas iki 2031 m.</t>
   </si>
   <si>
@@ -127,30 +148,9 @@
     <t xml:space="preserve">2026-06-29</t>
   </si>
   <si>
-    <t xml:space="preserve">Švietimas, mokslas ir sportas</t>
-  </si>
-  <si>
     <t xml:space="preserve">Pedagogų trūkumas ir kaita</t>
   </si>
   <si>
-    <t xml:space="preserve">STT nustatė korupcijos rizikas sporto infrastruktūros ir programų finansavime</t>
-  </si>
-  <si>
-    <t xml:space="preserve">„Per 2023–2025 m. iš valstybės biudžeto sporto finansavimui skirta daugiau kaip 76,6 mln. eurų.“ STT korupcijos rizikos analizė apėmė Švietimo, mokslo ir sporto ministeriją, Nacionalinę sporto agentūrą ir Vilniaus, Panevėžio, Kauno, Akmenės, Kupiškio bei Plungės savivaldybes. „Finansavimas skirtas futbolo klubui, kurio prezidentas buvo savivaldybės meras.“ Valstybės investuota baseinų infrastruktūra „naudojama ir komercinėmis SPA ar pirčių paslaugomis“ be aiškių viešojo intereso sąlygų.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">jp.lt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">jp.lt straipsnis</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-06-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sporto finansavimo skaidrumas ir interesų konfliktai</t>
-  </si>
-  <si>
     <t xml:space="preserve">Švietimo pagalba specialiųjų poreikių vaikams vėluoja dėl sisteminių spragų</t>
   </si>
   <si>
@@ -247,37 +247,37 @@
     <t xml:space="preserve">Civilinės saugos priedangų (slėptuvių) trūkumas</t>
   </si>
   <si>
+    <t xml:space="preserve">Klausimai dėl Vilniaus savivaldybės apmokamos komunikacijos su nuomonės formuotojais skaidrumo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">„Iš viso penkiems turinio kūrėjams skirta 6,8 tūkst. eurų be PVM, o daugiau nei pusė šios sumos – 3,8 tūkst. eurų – atiteko būtent R. Mackevičiui.“ Tarybos narys A. Nemunaitis: „Nieko kol kas nekaltinu – tam ir yra institucijos. Bet atsakymai į šiuos klausimus visuomenei turi būti pateikti.“ Kreiptasi į tris institucijas – Valstybinę vartotojų teisių apsaugos tarnybą, Vyriausiąją rinkimų komisiją ir Specialiųjų tyrimų tarnybą. „R. Mackevičiaus vaizdo įrašai surinko šimtus tūkstančių peržiūrų, o po kampanijos starto naujojo puslapio lankomumas išaugo daugiau nei vienuolika kartų.“</t>
+  </si>
+  <si>
+    <t xml:space="preserve">77.lt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">77.lt straipsnis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-04-21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Viešasis valdymas, regioninė politika ir viešasis administravimas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Savivaldybių komunikacijos ir viešųjų pirkimų skaidrumas</t>
+  </si>
+  <si>
     <t xml:space="preserve">Premjero žmonos įdarbinimas be konkurso Kauno r. savivaldybėje: nepotizmo kritika ir kontrolės institucijos spraga</t>
   </si>
   <si>
     <t xml:space="preserve">Aistė Sinkevičienė tapo Viešųjų ir tarptautinių ryšių skyriaus vedėja „be konkurso“ Kauno rajono savivaldybėje. Vienu metu dirbo tiek savivaldybėje, tiek Raudondvario dvare, tačiau žurnalistams „nepavyko rasti įrodymų, kad premjero žmona būtų faktiškai dirbusi, pavyzdžiui, Raudondvario dvare.“ S. Malinausko komentaras: „Visiškai akivaizdu, kad Raudondvaryje, Kauno rajono savivaldybėje turime švogerizmą, nepotizmą, darbo biržą, atidarytą saviems.“ Vėliau, komentuodama šią viešą diskusiją, „VDI teigia neturėjanti kompetencijos vertinti, ar valstybės ar savivaldybės įstaigoje dirbantis darbuotojas realiai atlieka savo pareigas“ – VDI nuomone, fiktyvaus įdarbinimo atvejų vertinimas turėtų priklausyti darbdaviui ir teisėsaugos institucijoms, o ne inspekcijai.</t>
   </si>
   <si>
-    <t xml:space="preserve">Viešasis valdymas, regioninė politika ir viešasis administravimas</t>
-  </si>
-  <si>
     <t xml:space="preserve">Nepotizmas ir personalo kontrolės institucinė spraga savivaldybėse</t>
   </si>
   <si>
     <t xml:space="preserve">2026-09-01 | LRT | https://www.lrt.lt/naujienos/lietuvoje/2/3038408/malinauskas-kauno-r-savivaldybeje-turime-svogerizma-nepotizma-darbo-birza-saviems  ;  2026-09-03 | 15min.lt | https://www.15min.lt/naujiena/aktualu/lietuva/vdi-teigia-kad-ne-jos-kompetencija-vertinti-ar-savivaldybes-istaigos-darbuotojas-realiai-dirba-56-2756030</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Klausimai dėl Vilniaus savivaldybės apmokamos komunikacijos su nuomonės formuotojais skaidrumo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">„Iš viso penkiems turinio kūrėjams skirta 6,8 tūkst. eurų be PVM, o daugiau nei pusė šios sumos – 3,8 tūkst. eurų – atiteko būtent R. Mackevičiui.“ Tarybos narys A. Nemunaitis: „Nieko kol kas nekaltinu – tam ir yra institucijos. Bet atsakymai į šiuos klausimus visuomenei turi būti pateikti.“ Kreiptasi į tris institucijas – Valstybinę vartotojų teisių apsaugos tarnybą, Vyriausiąją rinkimų komisiją ir Specialiųjų tyrimų tarnybą. „R. Mackevičiaus vaizdo įrašai surinko šimtus tūkstančių peržiūrų, o po kampanijos starto naujojo puslapio lankomumas išaugo daugiau nei vienuolika kartų.“</t>
-  </si>
-  <si>
-    <t xml:space="preserve">77.lt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">77.lt straipsnis</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04-21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Savivaldybių komunikacijos ir viešųjų pirkimų skaidrumas</t>
   </si>
 </sst>
 </file>
@@ -538,28 +538,28 @@
         <v>37</v>
       </c>
       <c r="D6" t="s" s="1">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="E6" t="s">
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="F6" t="s" s="1">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G6" t="s" s="1">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H6" t="s" s="1">
+        <v>42</v>
+      </c>
+      <c r="I6" t="s" s="1">
+        <v>18</v>
+      </c>
+      <c r="J6">
+        <v>1</v>
+      </c>
+      <c r="K6" t="s" s="1">
         <v>40</v>
-      </c>
-      <c r="I6" t="s" s="1">
-        <v>18</v>
-      </c>
-      <c r="J6">
-        <v>1</v>
-      </c>
-      <c r="K6" t="s" s="1">
-        <v>38</v>
       </c>
     </row>
     <row r="7">
@@ -567,22 +567,22 @@
         <v>6</v>
       </c>
       <c r="B7" t="s" s="1">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C7" t="s" s="1">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D7" t="s" s="1">
-        <v>43</v>
+        <v>26</v>
       </c>
       <c r="E7" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="F7" t="s" s="1">
         <v>45</v>
       </c>
       <c r="G7" t="s" s="1">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H7" t="s" s="1">
         <v>46</v>
@@ -617,7 +617,7 @@
         <v>51</v>
       </c>
       <c r="G8" t="s" s="1">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H8" t="s" s="1">
         <v>52</v>
@@ -783,28 +783,28 @@
         <v>80</v>
       </c>
       <c r="D13" t="s" s="1">
-        <v>26</v>
+        <v>81</v>
       </c>
       <c r="E13" t="s">
-        <v>27</v>
+        <v>82</v>
       </c>
       <c r="F13" t="s" s="1">
-        <v>15</v>
+        <v>83</v>
       </c>
       <c r="G13" t="s" s="1">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="H13" t="s" s="1">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="I13" t="s" s="1">
+        <v>18</v>
+      </c>
+      <c r="J13">
+        <v>1</v>
+      </c>
+      <c r="K13" t="s" s="1">
         <v>83</v>
-      </c>
-      <c r="J13">
-        <v>2</v>
-      </c>
-      <c r="K13" t="s" s="1">
-        <v>28</v>
       </c>
     </row>
     <row r="14">
@@ -812,34 +812,34 @@
         <v>13</v>
       </c>
       <c r="B14" t="s" s="1">
+        <v>86</v>
+      </c>
+      <c r="C14" t="s" s="1">
+        <v>87</v>
+      </c>
+      <c r="D14" t="s" s="1">
+        <v>26</v>
+      </c>
+      <c r="E14" t="s">
+        <v>27</v>
+      </c>
+      <c r="F14" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="G14" t="s" s="1">
         <v>84</v>
       </c>
-      <c r="C14" t="s" s="1">
-        <v>85</v>
-      </c>
-      <c r="D14" t="s" s="1">
-        <v>86</v>
-      </c>
-      <c r="E14" t="s">
-        <v>87</v>
-      </c>
-      <c r="F14" t="s" s="1">
+      <c r="H14" t="s" s="1">
         <v>88</v>
       </c>
-      <c r="G14" t="s" s="1">
-        <v>81</v>
-      </c>
-      <c r="H14" t="s" s="1">
+      <c r="I14" t="s" s="1">
         <v>89</v>
       </c>
-      <c r="I14" t="s" s="1">
-        <v>18</v>
-      </c>
       <c r="J14">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K14" t="s" s="1">
-        <v>88</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Savaitinis atnaujinimas 2026-09-03 (2-a banga): 2 naujos problemos, 82/96 šaltinių
- Elektros tinklo atkūrimas po audros (Energetika) — Anykšta, 2 paminėjimai
- 'Stasys Museum' lankytojų mažėjimas (Kultūra ir visuomenės informavimas) — Panevėžio kraštas
- Nauja sritis paliesta: Kultūra ir visuomenės informavimas (9/16 iš viso)

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ataskaitos/VK_zin_apzvalga_2026-09-03.xlsx
+++ b/ataskaitos/VK_zin_apzvalga_2026-09-03.xlsx
@@ -8,7 +8,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="103">
   <si>
     <t xml:space="preserve">Nr.</t>
   </si>
@@ -101,6 +101,45 @@
   </si>
   <si>
     <t xml:space="preserve">Elektros kainų nestabilumas ir priklausomybė nuo importo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Po galingiausios nuo 1970 m. audros elektros tinklas liko sugriautas, savivaldybių vadovai vengia komentuoti atkūrimo eigą</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Šio ryto duomenimis, šiek tiek virš 4 tūkst. [vartotojų] skirtingose šalies vietose neturi elektros energijos." "Blogiausia situacija ir toliau išlieka Utenos regione, taip pat Anykščių, Zarasų apylinkėse." "Tinklas iš tikrųjų yra sugriautas. Šita audra... buvo galingiausia nuo 1970 metų." "Kai kuriose vietovėse elektros tinklas yra taip stipriai pažeistas, jog šį reikės tiesti iš naujo." "Piko metu elektros tiekimas buvo sutrikęs daugiau kaip 268 tūkst. ESO klientų." Anykščių rajone užregistruoti "243 elektros tiekimo sutrikimai su 759 atjungtų klientų", atkūrimui dirbo "28 brigados... 11 skirtingų Anykščių rajono seniūnijų". Anykščių meras Kęstutis Tubis viešai atsakė trumpai: "Nebeturiu komentarų!!!"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anykšta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anykšta straipsnis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Elektros tinklų atkūrimas po stichinės nelaimės ir savivaldybių komunikacija</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-09-03 | Anykšta (ESO pranešimas) | https://www.anyksta.lt/eso-po-audros-elektros-vis-dar-neturi-per-4-tukst-vartotoju/  ;  2026-09-03 | Anykšta (mero komentaras) | https://www.anyksta.lt/meras-apie-elektra-nebeturiu-komentaru/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Panevėžio savivaldybės finansuojamas 'Stasys Museum' praranda lankytojus, savų pajamų dalis lieka minimali</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Pernai „Stasys Museum" apsilankė 70 591 lankytojas – tai net 12 239 lankytojais mažiau nei užpernai." Finansavimas: "beveik 2,3 mln. eurų – sudarė Panevėžio miesto savivaldybės biudžeto pinigai." "Muziejus pernai iš parduotų bilietų ir suteiktų paslaugų užsidirbo vos 114,5 tūkst. eurų, arba tik 4,35 procento." "Šių metų pirmąjį pusmetį „Stasys Museum" aplankė 34 645 lankytojai, vidutiniškai per mėnesį – beveik po 5800." Palyginimui, "per pirmąjį veiklos mėnesį užpraėjusią vasarą muziejus sulaukė beveik 20 tūkst. lankytojų."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Panevėžio kraštas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Panevėžio kraštas straipsnis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-08-28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kultūra ir visuomenės informavimas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Viešai finansuojamų kultūros įstaigų lankomumas ir savų pajamų dalis</t>
   </si>
   <si>
     <t xml:space="preserve">Klaipėdos miesto poliklinika per pusantrų metų neteko trečdalio gydytojų</t>
@@ -336,7 +375,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:K16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -503,28 +542,28 @@
         <v>32</v>
       </c>
       <c r="D5" t="s" s="1">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="E5" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="F5" t="s" s="1">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="G5" t="s" s="1">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="H5" t="s" s="1">
         <v>35</v>
       </c>
       <c r="I5" t="s" s="1">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="J5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K5" t="s" s="1">
-        <v>33</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6">
@@ -532,34 +571,34 @@
         <v>5</v>
       </c>
       <c r="B6" t="s" s="1">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C6" t="s" s="1">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D6" t="s" s="1">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F6" t="s" s="1">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G6" t="s" s="1">
+        <v>42</v>
+      </c>
+      <c r="H6" t="s" s="1">
+        <v>43</v>
+      </c>
+      <c r="I6" t="s" s="1">
+        <v>18</v>
+      </c>
+      <c r="J6">
+        <v>1</v>
+      </c>
+      <c r="K6" t="s" s="1">
         <v>41</v>
-      </c>
-      <c r="H6" t="s" s="1">
-        <v>42</v>
-      </c>
-      <c r="I6" t="s" s="1">
-        <v>18</v>
-      </c>
-      <c r="J6">
-        <v>1</v>
-      </c>
-      <c r="K6" t="s" s="1">
-        <v>40</v>
       </c>
     </row>
     <row r="7">
@@ -567,34 +606,34 @@
         <v>6</v>
       </c>
       <c r="B7" t="s" s="1">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C7" t="s" s="1">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D7" t="s" s="1">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="E7" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="F7" t="s" s="1">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G7" t="s" s="1">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="H7" t="s" s="1">
+        <v>48</v>
+      </c>
+      <c r="I7" t="s" s="1">
+        <v>18</v>
+      </c>
+      <c r="J7">
+        <v>1</v>
+      </c>
+      <c r="K7" t="s" s="1">
         <v>46</v>
-      </c>
-      <c r="I7" t="s" s="1">
-        <v>18</v>
-      </c>
-      <c r="J7">
-        <v>1</v>
-      </c>
-      <c r="K7" t="s" s="1">
-        <v>45</v>
       </c>
     </row>
     <row r="8">
@@ -602,34 +641,34 @@
         <v>7</v>
       </c>
       <c r="B8" t="s" s="1">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C8" t="s" s="1">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D8" t="s" s="1">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E8" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F8" t="s" s="1">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="G8" t="s" s="1">
-        <v>41</v>
+        <v>54</v>
       </c>
       <c r="H8" t="s" s="1">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="I8" t="s" s="1">
+        <v>18</v>
+      </c>
+      <c r="J8">
+        <v>1</v>
+      </c>
+      <c r="K8" t="s" s="1">
         <v>53</v>
-      </c>
-      <c r="J8">
-        <v>3</v>
-      </c>
-      <c r="K8" t="s" s="1">
-        <v>54</v>
       </c>
     </row>
     <row r="9">
@@ -637,22 +676,22 @@
         <v>8</v>
       </c>
       <c r="B9" t="s" s="1">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C9" t="s" s="1">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D9" t="s" s="1">
-        <v>49</v>
+        <v>26</v>
       </c>
       <c r="E9" t="s">
-        <v>50</v>
+        <v>27</v>
       </c>
       <c r="F9" t="s" s="1">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G9" t="s" s="1">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="H9" t="s" s="1">
         <v>59</v>
@@ -664,7 +703,7 @@
         <v>1</v>
       </c>
       <c r="K9" t="s" s="1">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="10">
@@ -684,22 +723,22 @@
         <v>63</v>
       </c>
       <c r="F10" t="s" s="1">
-        <v>15</v>
+        <v>64</v>
       </c>
       <c r="G10" t="s" s="1">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="H10" t="s" s="1">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="I10" t="s" s="1">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="J10">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K10" t="s" s="1">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="11">
@@ -707,34 +746,34 @@
         <v>10</v>
       </c>
       <c r="B11" t="s" s="1">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C11" t="s" s="1">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D11" t="s" s="1">
-        <v>13</v>
+        <v>62</v>
       </c>
       <c r="E11" t="s">
-        <v>14</v>
+        <v>63</v>
       </c>
       <c r="F11" t="s" s="1">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="G11" t="s" s="1">
+        <v>71</v>
+      </c>
+      <c r="H11" t="s" s="1">
+        <v>72</v>
+      </c>
+      <c r="I11" t="s" s="1">
+        <v>18</v>
+      </c>
+      <c r="J11">
+        <v>1</v>
+      </c>
+      <c r="K11" t="s" s="1">
         <v>70</v>
-      </c>
-      <c r="H11" t="s" s="1">
-        <v>71</v>
-      </c>
-      <c r="I11" t="s" s="1">
-        <v>18</v>
-      </c>
-      <c r="J11">
-        <v>1</v>
-      </c>
-      <c r="K11" t="s" s="1">
-        <v>69</v>
       </c>
     </row>
     <row r="12">
@@ -742,34 +781,34 @@
         <v>11</v>
       </c>
       <c r="B12" t="s" s="1">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C12" t="s" s="1">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D12" t="s" s="1">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E12" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F12" t="s" s="1">
-        <v>76</v>
+        <v>15</v>
       </c>
       <c r="G12" t="s" s="1">
+        <v>71</v>
+      </c>
+      <c r="H12" t="s" s="1">
         <v>77</v>
       </c>
-      <c r="H12" t="s" s="1">
+      <c r="I12" t="s" s="1">
         <v>78</v>
       </c>
-      <c r="I12" t="s" s="1">
-        <v>18</v>
-      </c>
       <c r="J12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K12" t="s" s="1">
-        <v>76</v>
+        <v>79</v>
       </c>
     </row>
     <row r="13">
@@ -777,26 +816,26 @@
         <v>12</v>
       </c>
       <c r="B13" t="s" s="1">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C13" t="s" s="1">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D13" t="s" s="1">
-        <v>81</v>
+        <v>13</v>
       </c>
       <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s" s="1">
         <v>82</v>
       </c>
-      <c r="F13" t="s" s="1">
+      <c r="G13" t="s" s="1">
         <v>83</v>
       </c>
-      <c r="G13" t="s" s="1">
+      <c r="H13" t="s" s="1">
         <v>84</v>
       </c>
-      <c r="H13" t="s" s="1">
-        <v>85</v>
-      </c>
       <c r="I13" t="s" s="1">
         <v>18</v>
       </c>
@@ -804,7 +843,7 @@
         <v>1</v>
       </c>
       <c r="K13" t="s" s="1">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="14">
@@ -812,38 +851,108 @@
         <v>13</v>
       </c>
       <c r="B14" t="s" s="1">
+        <v>85</v>
+      </c>
+      <c r="C14" t="s" s="1">
         <v>86</v>
       </c>
-      <c r="C14" t="s" s="1">
+      <c r="D14" t="s" s="1">
         <v>87</v>
       </c>
-      <c r="D14" t="s" s="1">
+      <c r="E14" t="s">
+        <v>88</v>
+      </c>
+      <c r="F14" t="s" s="1">
+        <v>89</v>
+      </c>
+      <c r="G14" t="s" s="1">
+        <v>90</v>
+      </c>
+      <c r="H14" t="s" s="1">
+        <v>91</v>
+      </c>
+      <c r="I14" t="s" s="1">
+        <v>18</v>
+      </c>
+      <c r="J14">
+        <v>1</v>
+      </c>
+      <c r="K14" t="s" s="1">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s" s="1">
+        <v>92</v>
+      </c>
+      <c r="C15" t="s" s="1">
+        <v>93</v>
+      </c>
+      <c r="D15" t="s" s="1">
+        <v>94</v>
+      </c>
+      <c r="E15" t="s">
+        <v>95</v>
+      </c>
+      <c r="F15" t="s" s="1">
+        <v>96</v>
+      </c>
+      <c r="G15" t="s" s="1">
+        <v>97</v>
+      </c>
+      <c r="H15" t="s" s="1">
+        <v>98</v>
+      </c>
+      <c r="I15" t="s" s="1">
+        <v>18</v>
+      </c>
+      <c r="J15">
+        <v>1</v>
+      </c>
+      <c r="K15" t="s" s="1">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s" s="1">
+        <v>99</v>
+      </c>
+      <c r="C16" t="s" s="1">
+        <v>100</v>
+      </c>
+      <c r="D16" t="s" s="1">
         <v>26</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E16" t="s">
         <v>27</v>
       </c>
-      <c r="F14" t="s" s="1">
+      <c r="F16" t="s" s="1">
         <v>15</v>
       </c>
-      <c r="G14" t="s" s="1">
-        <v>84</v>
-      </c>
-      <c r="H14" t="s" s="1">
-        <v>88</v>
-      </c>
-      <c r="I14" t="s" s="1">
-        <v>89</v>
-      </c>
-      <c r="J14">
+      <c r="G16" t="s" s="1">
+        <v>97</v>
+      </c>
+      <c r="H16" t="s" s="1">
+        <v>101</v>
+      </c>
+      <c r="I16" t="s" s="1">
+        <v>102</v>
+      </c>
+      <c r="J16">
         <v>2</v>
       </c>
-      <c r="K14" t="s" s="1">
+      <c r="K16" t="s" s="1">
         <v>28</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K14"/>
+  <autoFilter ref="A1:K16"/>
   <hyperlinks>
     <hyperlink ref="E2" r:id="rIdHL1"/>
     <hyperlink ref="E3" r:id="rIdHL2"/>
@@ -858,6 +967,8 @@
     <hyperlink ref="E12" r:id="rIdHL11"/>
     <hyperlink ref="E13" r:id="rIdHL12"/>
     <hyperlink ref="E14" r:id="rIdHL13"/>
+    <hyperlink ref="E15" r:id="rIdHL14"/>
+    <hyperlink ref="E16" r:id="rIdHL15"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>